<commit_message>
Update core templates and backend with current data snapshots.
Refresh sales, schedule, and related pages, and commit project data JSON including dispatch remarks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/uploads/차량정비_2026.xlsx
+++ b/uploads/차량정비_2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\HanMi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pdata\ojy-hmtaxi-erp\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0B2338-B48C-4EDA-9D06-5B9A77993E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C27FDE-7137-4ED4-BD4D-54C685F0A6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="216" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{523E7D56-C0C9-4D7D-B9FB-0F40CB567697}"/>
+    <workbookView xWindow="22932" yWindow="216" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{523E7D56-C0C9-4D7D-B9FB-0F40CB567697}"/>
   </bookViews>
   <sheets>
     <sheet name="1월" sheetId="11" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="39">
   <si>
     <t>차번</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -52,10 +52,6 @@
   </si>
   <si>
     <t>검사</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>타이어교체</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -124,10 +120,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>타이어_펑크</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>○</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -145,6 +137,52 @@
   </si>
   <si>
     <t>m</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>m</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예방정비(7/23)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>리콜A/S(현대당산점)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>△</t>
+  </si>
+  <si>
+    <t>□</t>
+  </si>
+  <si>
+    <t>타이어파스, 서교동출장수리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예방정비(8/06)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>△</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예방정비(8/03)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예방정비(8/05)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>□</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1157,19 +1195,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -1181,22 +1219,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -1215,7 +1253,7 @@
         <v>45966</v>
       </c>
       <c r="M2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -1234,7 +1272,7 @@
         <v>45966</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I3" s="8">
         <v>2</v>
@@ -1256,7 +1294,7 @@
         <v>45873</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I4" s="8">
         <v>2</v>
@@ -1278,7 +1316,7 @@
         <v>44655</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -1297,7 +1335,7 @@
         <v>44636</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I6" s="8">
         <v>2</v>
@@ -1319,7 +1357,7 @@
         <v>44756</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1338,7 +1376,7 @@
         <v>44316</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1357,7 +1395,7 @@
         <v>45455</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="K9" s="8">
         <v>1</v>
@@ -1379,7 +1417,7 @@
         <v>44609</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1398,7 +1436,7 @@
         <v>45166</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I11" s="8">
         <v>2</v>
@@ -1439,7 +1477,7 @@
         <v>44566</v>
       </c>
       <c r="M13" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -1458,7 +1496,7 @@
         <v>44566</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I14" s="8">
         <v>3</v>
@@ -1480,7 +1518,7 @@
         <v>45477</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I15" s="8">
         <v>2</v>
@@ -1502,7 +1540,7 @@
         <v>45477</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -1521,7 +1559,7 @@
         <v>45602</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
@@ -1540,7 +1578,7 @@
         <v>44288</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -2705,19 +2743,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -2729,22 +2767,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -4100,19 +4138,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -4124,22 +4162,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -5498,19 +5536,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -5522,22 +5560,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -6880,10 +6918,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -6891,7 +6929,7 @@
         <v>1801</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="4">
         <v>45966</v>
@@ -6903,7 +6941,7 @@
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -6911,7 +6949,7 @@
         <v>1803</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="5">
         <v>44566</v>
@@ -6922,7 +6960,7 @@
         <v>1804</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5">
         <v>45873</v>
@@ -6934,7 +6972,7 @@
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -6942,7 +6980,7 @@
         <v>1807</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="5">
         <v>44288</v>
@@ -6954,7 +6992,7 @@
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -6962,7 +7000,7 @@
         <v>1809</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="5">
         <v>45615</v>
@@ -6974,7 +7012,7 @@
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -6982,7 +7020,7 @@
         <v>1812</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="5">
         <v>45594</v>
@@ -6993,7 +7031,7 @@
         <v>1813</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="5">
         <v>45166</v>
@@ -7004,7 +7042,7 @@
         <v>1814</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="5">
         <v>45626</v>
@@ -7015,7 +7053,7 @@
         <v>1815</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" s="5">
         <v>45626</v>
@@ -7027,7 +7065,7 @@
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -7036,7 +7074,7 @@
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -7045,7 +7083,7 @@
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -7053,7 +7091,7 @@
         <v>1819</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C18" s="5">
         <v>45873</v>
@@ -7065,7 +7103,7 @@
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -7074,7 +7112,7 @@
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -7082,7 +7120,7 @@
         <v>1823</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C21" s="5">
         <v>45455</v>
@@ -7093,7 +7131,7 @@
         <v>1825</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22" s="5">
         <v>45626</v>
@@ -7104,7 +7142,7 @@
         <v>1826</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C23" s="5">
         <v>44802</v>
@@ -7116,7 +7154,7 @@
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -7124,7 +7162,7 @@
         <v>1828</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C25" s="5">
         <v>44566</v>
@@ -7136,7 +7174,7 @@
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -7144,7 +7182,7 @@
         <v>1830</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C27" s="5">
         <v>45966</v>
@@ -7155,7 +7193,7 @@
         <v>1832</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" s="5">
         <v>44609</v>
@@ -7166,7 +7204,7 @@
         <v>1833</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C29" s="5">
         <v>45904</v>
@@ -7178,7 +7216,7 @@
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -7186,7 +7224,7 @@
         <v>1835</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" s="5">
         <v>45547</v>
@@ -7197,7 +7235,7 @@
         <v>1836</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="5">
         <v>45931</v>
@@ -7209,7 +7247,7 @@
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -7217,7 +7255,7 @@
         <v>1839</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C34" s="5">
         <v>44802</v>
@@ -7228,7 +7266,7 @@
         <v>1840</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C35" s="5">
         <v>45477</v>
@@ -7239,7 +7277,7 @@
         <v>1842</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="5">
         <v>45594</v>
@@ -7250,7 +7288,7 @@
         <v>1843</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C37" s="5">
         <v>45974</v>
@@ -7261,10 +7299,10 @@
         <v>1844</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -7273,7 +7311,7 @@
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -7281,7 +7319,7 @@
         <v>1847</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C40" s="5">
         <v>45534</v>
@@ -7292,7 +7330,7 @@
         <v>1848</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41" s="5">
         <v>44802</v>
@@ -7303,7 +7341,7 @@
         <v>1849</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C42" s="5">
         <v>44804</v>
@@ -7314,7 +7352,7 @@
         <v>1850</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C43" s="5">
         <v>45957</v>
@@ -7325,7 +7363,7 @@
         <v>1852</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C44" s="5">
         <v>44655</v>
@@ -7336,7 +7374,7 @@
         <v>1853</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C45" s="5">
         <v>44609</v>
@@ -7347,7 +7385,7 @@
         <v>1856</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C46" s="5">
         <v>45959</v>
@@ -7358,7 +7396,7 @@
         <v>1857</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C47" s="5">
         <v>45904</v>
@@ -7369,7 +7407,7 @@
         <v>1858</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C48" s="5">
         <v>45959</v>
@@ -7380,7 +7418,7 @@
         <v>1859</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C49" s="5">
         <v>45096</v>
@@ -7392,7 +7430,7 @@
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -7400,7 +7438,7 @@
         <v>1862</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C51" s="5">
         <v>45565</v>
@@ -7411,7 +7449,7 @@
         <v>1863</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C52" s="5">
         <v>45594</v>
@@ -7422,7 +7460,7 @@
         <v>1865</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C53" s="5">
         <v>44516</v>
@@ -7433,7 +7471,7 @@
         <v>1866</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C54" s="5">
         <v>45602</v>
@@ -7445,7 +7483,7 @@
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -7453,7 +7491,7 @@
         <v>1868</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C56" s="5">
         <v>45216</v>
@@ -7464,7 +7502,7 @@
         <v>1869</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C57" s="5">
         <v>45216</v>
@@ -7475,7 +7513,7 @@
         <v>1870</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C58" s="5">
         <v>45594</v>
@@ -7486,7 +7524,7 @@
         <v>1871</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C59" s="5">
         <v>45602</v>
@@ -7497,7 +7535,7 @@
         <v>1872</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C60" s="5">
         <v>45966</v>
@@ -7509,7 +7547,7 @@
       </c>
       <c r="B61" s="3"/>
       <c r="C61" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -7517,7 +7555,7 @@
         <v>1874</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C62" s="5">
         <v>45974</v>
@@ -7529,7 +7567,7 @@
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -7537,7 +7575,7 @@
         <v>1876</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C64" s="5">
         <v>45547</v>
@@ -7548,7 +7586,7 @@
         <v>1877</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C65" s="5">
         <v>45610</v>
@@ -7559,7 +7597,7 @@
         <v>1878</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C66" s="5">
         <v>45632</v>
@@ -7570,7 +7608,7 @@
         <v>1879</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C67" s="5">
         <v>44804</v>
@@ -7581,7 +7619,7 @@
         <v>1880</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C68" s="5">
         <v>45632</v>
@@ -7592,7 +7630,7 @@
         <v>1881</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C69" s="5">
         <v>44804</v>
@@ -7604,7 +7642,7 @@
       </c>
       <c r="B70" s="3"/>
       <c r="C70" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -7612,7 +7650,7 @@
         <v>1883</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C71" s="5">
         <v>45455</v>
@@ -7624,7 +7662,7 @@
       </c>
       <c r="B72" s="3"/>
       <c r="C72" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -7632,7 +7670,7 @@
         <v>1886</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C73" s="5">
         <v>44529</v>
@@ -7643,7 +7681,7 @@
         <v>1888</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C74" s="5">
         <v>45974</v>
@@ -7654,7 +7692,7 @@
         <v>1889</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C75" s="5">
         <v>44777</v>
@@ -7665,7 +7703,7 @@
         <v>1890</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C76" s="5">
         <v>44636</v>
@@ -7677,7 +7715,7 @@
       </c>
       <c r="B77" s="3"/>
       <c r="C77" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -7685,7 +7723,7 @@
         <v>1893</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C78" s="5">
         <v>44552</v>
@@ -7696,7 +7734,7 @@
         <v>1894</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C79" s="5">
         <v>44552</v>
@@ -7707,7 +7745,7 @@
         <v>1895</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C80" s="5">
         <v>44558</v>
@@ -7718,7 +7756,7 @@
         <v>1896</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C81" s="5">
         <v>45229</v>
@@ -7730,7 +7768,7 @@
       </c>
       <c r="B82" s="3"/>
       <c r="C82" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -7738,7 +7776,7 @@
         <v>1898</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C83" s="5">
         <v>45547</v>
@@ -7750,7 +7788,7 @@
       </c>
       <c r="B84" s="3"/>
       <c r="C84" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -7758,7 +7796,7 @@
         <v>1900</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C85" s="5">
         <v>44655</v>
@@ -7769,7 +7807,7 @@
         <v>1901</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C86" s="5">
         <v>45477</v>
@@ -7780,7 +7818,7 @@
         <v>1902</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C87" s="5">
         <v>44756</v>
@@ -7791,7 +7829,7 @@
         <v>1903</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C88" s="5">
         <v>44777</v>
@@ -7802,7 +7840,7 @@
         <v>1904</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C89" s="5">
         <v>45477</v>
@@ -7814,7 +7852,7 @@
       </c>
       <c r="B90" s="3"/>
       <c r="C90" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -7823,7 +7861,7 @@
       </c>
       <c r="B91" s="3"/>
       <c r="C91" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -7831,7 +7869,7 @@
         <v>1908</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C92" s="5">
         <v>45904</v>
@@ -7842,7 +7880,7 @@
         <v>1911</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C93" s="5">
         <v>45602</v>
@@ -7853,7 +7891,7 @@
         <v>1912</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C94" s="5">
         <v>45455</v>
@@ -7865,7 +7903,7 @@
       </c>
       <c r="B95" s="3"/>
       <c r="C95" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -7873,7 +7911,7 @@
         <v>1915</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C96" s="5">
         <v>44316</v>
@@ -7884,7 +7922,7 @@
         <v>7631</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
@@ -7892,7 +7930,7 @@
         <v>7632</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -7900,7 +7938,7 @@
         <v>7633</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -7908,7 +7946,7 @@
         <v>7634</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -7916,7 +7954,7 @@
         <v>7635</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -7924,7 +7962,7 @@
         <v>7636</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -7932,7 +7970,7 @@
         <v>7637</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -7940,7 +7978,7 @@
         <v>7638</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -7948,7 +7986,7 @@
         <v>7639</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -7956,7 +7994,7 @@
         <v>7640</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -7991,19 +8029,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -8015,22 +8053,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -8049,7 +8087,7 @@
         <v>45966</v>
       </c>
       <c r="M2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -8068,7 +8106,7 @@
         <v>44566</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -8087,7 +8125,7 @@
         <v>45873</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -8106,7 +8144,7 @@
         <v>45873</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J5" s="8">
         <v>2</v>
@@ -8128,7 +8166,7 @@
         <v>44566</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -8147,7 +8185,7 @@
         <v>45477</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K7" s="8">
         <v>1</v>
@@ -8169,7 +8207,7 @@
         <v>44288</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -8188,7 +8226,7 @@
         <v>45166</v>
       </c>
       <c r="M9" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -8207,7 +8245,7 @@
         <v>45626</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N10" s="14"/>
     </row>
@@ -8227,7 +8265,7 @@
         <v>45632</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L11" s="8">
         <v>1</v>
@@ -8249,7 +8287,7 @@
         <v>45966</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I12" s="8">
         <v>5</v>
@@ -8271,7 +8309,7 @@
         <v>45166</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I13" s="8">
         <v>4</v>
@@ -8293,7 +8331,7 @@
         <v>45602</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K14" s="8">
         <v>1</v>
@@ -8315,7 +8353,7 @@
         <v>45602</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -8334,7 +8372,7 @@
         <v>45626</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -8353,7 +8391,7 @@
         <v>45873</v>
       </c>
       <c r="M17" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
@@ -8372,7 +8410,7 @@
         <v>45455</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -8391,7 +8429,7 @@
         <v>45455</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I19" s="8">
         <v>2</v>
@@ -8413,7 +8451,7 @@
         <v>45904</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
@@ -8432,10 +8470,10 @@
         <v>45547</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
@@ -8454,7 +8492,7 @@
         <v>45626</v>
       </c>
       <c r="M22" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
@@ -8473,7 +8511,7 @@
         <v>44566</v>
       </c>
       <c r="M23" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
@@ -8492,7 +8530,7 @@
         <v>45966</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
@@ -9575,19 +9613,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -9599,22 +9637,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -10970,19 +11008,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -10994,22 +11032,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -12365,19 +12403,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -12389,22 +12427,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -13760,19 +13798,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -13784,22 +13822,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -15155,19 +15193,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -15179,22 +15217,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -16529,7 +16567,7 @@
   <dimension ref="A1:N150"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.125" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.375" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.375" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.125" style="9" bestFit="1" customWidth="1"/>
@@ -16540,7 +16578,7 @@
     <col min="9" max="10" width="11.25" style="8" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="11" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.25" style="19" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.25" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.625" style="8" bestFit="1" customWidth="1"/>
     <col min="15" max="20" width="9.75" style="8" customWidth="1"/>
     <col min="21" max="21" width="11" style="8" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="7.125" style="8" bestFit="1" customWidth="1"/>
@@ -16550,19 +16588,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -16574,26 +16612,28 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
-        <v>17</v>
-      </c>
       <c r="K1" s="8" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>20</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="9"/>
+      <c r="A2" s="9">
+        <v>46235</v>
+      </c>
       <c r="B2" s="10"/>
       <c r="C2" s="11" t="str">
         <f>IFERROR(VLOOKUP(B2,차량리스트!$A:$C,2,0),"")</f>
@@ -16603,354 +16643,603 @@
         <f>IFERROR(VLOOKUP(B2,차량리스트!$A:$C,3,0),"")</f>
         <v/>
       </c>
+      <c r="I2" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="9">
+        <v>46236</v>
+      </c>
+      <c r="B3" s="13">
+        <v>1801</v>
+      </c>
       <c r="C3" s="11" t="str">
         <f>IFERROR(VLOOKUP(B3,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D3" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D3" s="12">
         <f>IFERROR(VLOOKUP(B3,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45966</v>
+      </c>
+      <c r="M3" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="9">
+        <v>46236</v>
+      </c>
+      <c r="B4" s="13">
+        <v>1803</v>
+      </c>
       <c r="C4" s="11" t="str">
         <f>IFERROR(VLOOKUP(B4,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D4" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D4" s="12">
         <f>IFERROR(VLOOKUP(B4,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>44566</v>
+      </c>
+      <c r="M4" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="13"/>
+      <c r="A5" s="9">
+        <v>46237</v>
+      </c>
+      <c r="B5" s="13">
+        <v>1801</v>
+      </c>
       <c r="C5" s="11" t="str">
         <f>IFERROR(VLOOKUP(B5,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D5" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D5" s="12">
         <f>IFERROR(VLOOKUP(B5,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45966</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="8">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="9">
+        <v>46237</v>
+      </c>
+      <c r="B6" s="13">
+        <v>1890</v>
+      </c>
       <c r="C6" s="11" t="str">
         <f>IFERROR(VLOOKUP(B6,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D6" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D6" s="12">
         <f>IFERROR(VLOOKUP(B6,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>44636</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="13"/>
+      <c r="A7" s="9">
+        <v>46237</v>
+      </c>
+      <c r="B7" s="13">
+        <v>1804</v>
+      </c>
       <c r="C7" s="11" t="str">
         <f>IFERROR(VLOOKUP(B7,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D7" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D7" s="12">
         <f>IFERROR(VLOOKUP(B7,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45873</v>
+      </c>
+      <c r="M7" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="13"/>
+      <c r="A8" s="9">
+        <v>46237</v>
+      </c>
+      <c r="B8" s="13">
+        <v>1813</v>
+      </c>
       <c r="C8" s="11" t="str">
         <f>IFERROR(VLOOKUP(B8,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D8" s="12">
         <f>IFERROR(VLOOKUP(B8,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45166</v>
+      </c>
+      <c r="M8" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="13"/>
+      <c r="A9" s="9">
+        <v>46237</v>
+      </c>
+      <c r="B9" s="13">
+        <v>1880</v>
+      </c>
       <c r="C9" s="11" t="str">
         <f>IFERROR(VLOOKUP(B9,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D9" s="12" t="str">
+        <v>아닉</v>
+      </c>
+      <c r="D9" s="12">
         <f>IFERROR(VLOOKUP(B9,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45632</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="13"/>
+      <c r="A10" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B10" s="13">
+        <v>1804</v>
+      </c>
       <c r="C10" s="11" t="str">
         <f>IFERROR(VLOOKUP(B10,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D10" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D10" s="12">
         <f>IFERROR(VLOOKUP(B10,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45873</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="8">
+        <v>2</v>
       </c>
       <c r="N10" s="14"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="13"/>
+      <c r="A11" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B11" s="13">
+        <v>1813</v>
+      </c>
       <c r="C11" s="11" t="str">
         <f>IFERROR(VLOOKUP(B11,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D11" s="12">
         <f>IFERROR(VLOOKUP(B11,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45166</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="13"/>
+      <c r="A12" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B12" s="13">
+        <v>1840</v>
+      </c>
       <c r="C12" s="11" t="str">
         <f>IFERROR(VLOOKUP(B12,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D12" s="12">
         <f>IFERROR(VLOOKUP(B12,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45477</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="13"/>
+      <c r="A13" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B13" s="13">
+        <v>1868</v>
+      </c>
       <c r="C13" s="11" t="str">
         <f>IFERROR(VLOOKUP(B13,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D13" s="12">
         <f>IFERROR(VLOOKUP(B13,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45216</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="13"/>
+      <c r="A14" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B14" s="13">
+        <v>1833</v>
+      </c>
       <c r="C14" s="11" t="str">
         <f>IFERROR(VLOOKUP(B14,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D14" s="12">
         <f>IFERROR(VLOOKUP(B14,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45904</v>
+      </c>
+      <c r="K14" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="13"/>
+      <c r="A15" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B15" s="13">
+        <v>1814</v>
+      </c>
       <c r="C15" s="11" t="str">
         <f>IFERROR(VLOOKUP(B15,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="12" t="str">
+        <v>쏘타</v>
+      </c>
+      <c r="D15" s="12">
         <f>IFERROR(VLOOKUP(B15,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>45626</v>
+      </c>
+      <c r="M15" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="13"/>
+      <c r="A16" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B16" s="13">
+        <v>1815</v>
+      </c>
       <c r="C16" s="11" t="str">
         <f>IFERROR(VLOOKUP(B16,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="12" t="str">
+        <v>쏘타</v>
+      </c>
+      <c r="D16" s="12">
         <f>IFERROR(VLOOKUP(B16,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="13"/>
+        <v>45626</v>
+      </c>
+      <c r="M16" s="19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="9">
+        <v>46238</v>
+      </c>
+      <c r="B17" s="13">
+        <v>1902</v>
+      </c>
       <c r="C17" s="11" t="str">
         <f>IFERROR(VLOOKUP(B17,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="12" t="str">
+        <v>니로</v>
+      </c>
+      <c r="D17" s="12">
         <f>IFERROR(VLOOKUP(B17,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="13"/>
+        <v>44756</v>
+      </c>
+      <c r="N17" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B18" s="13">
+        <v>1819</v>
+      </c>
       <c r="C18" s="11" t="str">
         <f>IFERROR(VLOOKUP(B18,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D18" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D18" s="12">
         <f>IFERROR(VLOOKUP(B18,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="13"/>
+        <v>45873</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="N18" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B19" s="13">
+        <v>1812</v>
+      </c>
       <c r="C19" s="11" t="str">
         <f>IFERROR(VLOOKUP(B19,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="12" t="str">
+        <v>아닉</v>
+      </c>
+      <c r="D19" s="12">
         <f>IFERROR(VLOOKUP(B19,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="13"/>
+        <v>45594</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B20" s="13">
+        <v>1826</v>
+      </c>
       <c r="C20" s="11" t="str">
         <f>IFERROR(VLOOKUP(B20,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D20" s="12" t="str">
+        <v>니로</v>
+      </c>
+      <c r="D20" s="12">
         <f>IFERROR(VLOOKUP(B20,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="13"/>
+        <v>44802</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B21" s="13">
+        <v>1835</v>
+      </c>
       <c r="C21" s="11" t="str">
         <f>IFERROR(VLOOKUP(B21,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="12" t="str">
+        <v>아닉</v>
+      </c>
+      <c r="D21" s="12">
         <f>IFERROR(VLOOKUP(B21,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="13"/>
+        <v>45547</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B22" s="13">
+        <v>1826</v>
+      </c>
       <c r="C22" s="11" t="str">
         <f>IFERROR(VLOOKUP(B22,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="12" t="str">
+        <v>니로</v>
+      </c>
+      <c r="D22" s="12">
         <f>IFERROR(VLOOKUP(B22,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="13"/>
+        <v>44802</v>
+      </c>
+      <c r="K22" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B23" s="13">
+        <v>1835</v>
+      </c>
       <c r="C23" s="11" t="str">
         <f>IFERROR(VLOOKUP(B23,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D23" s="12" t="str">
+        <v>아닉</v>
+      </c>
+      <c r="D23" s="12">
         <f>IFERROR(VLOOKUP(B23,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="13"/>
+        <v>45547</v>
+      </c>
+      <c r="K23" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A24" s="9">
+        <v>46239</v>
+      </c>
+      <c r="B24" s="13">
+        <v>1825</v>
+      </c>
       <c r="C24" s="11" t="str">
         <f>IFERROR(VLOOKUP(B24,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D24" s="12" t="str">
+        <v>쏘타</v>
+      </c>
+      <c r="D24" s="12">
         <f>IFERROR(VLOOKUP(B24,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="13"/>
+        <v>45626</v>
+      </c>
+      <c r="M24" s="19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B25" s="13">
+        <v>1803</v>
+      </c>
       <c r="C25" s="11" t="str">
         <f>IFERROR(VLOOKUP(B25,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D25" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D25" s="12">
         <f>IFERROR(VLOOKUP(B25,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="13"/>
+        <v>44566</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I25" s="8">
+        <v>2</v>
+      </c>
+      <c r="N25" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B26" s="13">
+        <v>1815</v>
+      </c>
       <c r="C26" s="11" t="str">
         <f>IFERROR(VLOOKUP(B26,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D26" s="12" t="str">
+        <v>쏘타</v>
+      </c>
+      <c r="D26" s="12">
         <f>IFERROR(VLOOKUP(B26,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="13"/>
+        <v>45626</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="N26" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B27" s="13">
+        <v>1825</v>
+      </c>
       <c r="C27" s="11" t="str">
         <f>IFERROR(VLOOKUP(B27,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D27" s="12" t="str">
+        <v>쏘타</v>
+      </c>
+      <c r="D27" s="12">
         <f>IFERROR(VLOOKUP(B27,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="13"/>
+        <v>45626</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B28" s="13">
+        <v>1868</v>
+      </c>
       <c r="C28" s="11" t="str">
         <f>IFERROR(VLOOKUP(B28,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D28" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D28" s="12">
         <f>IFERROR(VLOOKUP(B28,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="13"/>
+        <v>45216</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B29" s="13">
+        <v>1888</v>
+      </c>
       <c r="C29" s="11" t="str">
         <f>IFERROR(VLOOKUP(B29,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D29" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D29" s="12">
         <f>IFERROR(VLOOKUP(B29,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="13"/>
+        <v>45974</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B30" s="13">
+        <v>1813</v>
+      </c>
       <c r="C30" s="11" t="str">
         <f>IFERROR(VLOOKUP(B30,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D30" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D30" s="12">
         <f>IFERROR(VLOOKUP(B30,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B31" s="13"/>
+        <v>45166</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B31" s="13">
+        <v>1830</v>
+      </c>
       <c r="C31" s="11" t="str">
         <f>IFERROR(VLOOKUP(B31,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D31" s="12" t="str">
+        <v>K5</v>
+      </c>
+      <c r="D31" s="12">
         <f>IFERROR(VLOOKUP(B31,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="13"/>
+        <v>45966</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="9">
+        <v>46240</v>
+      </c>
+      <c r="B32" s="13">
+        <v>1832</v>
+      </c>
       <c r="C32" s="11" t="str">
         <f>IFERROR(VLOOKUP(B32,차량리스트!$A:$C,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="12" t="str">
+        <v>K5H</v>
+      </c>
+      <c r="D32" s="12">
         <f>IFERROR(VLOOKUP(B32,차량리스트!$A:$C,3,0),"")</f>
-        <v/>
+        <v>44609</v>
+      </c>
+      <c r="M32" s="19" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
@@ -17945,19 +18234,19 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -17969,22 +18258,22 @@
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>